<commit_message>
Updated: Test cases with new logic
</commit_message>
<xml_diff>
--- a/APPT/data/output/Final_Production_Plan_2026-01-13.xlsx
+++ b/APPT/data/output/Final_Production_Plan_2026-01-13.xlsx
@@ -267,49 +267,88 @@
     <t>H&amp;S CM</t>
   </si>
   <si>
-    <t>CI463</t>
+    <t>CI467</t>
   </si>
   <si>
     <t>REP01-0113</t>
   </si>
   <si>
-    <t>CI464</t>
-  </si>
-  <si>
-    <t>CI465</t>
-  </si>
-  <si>
-    <t>CI467</t>
+    <t>CI468</t>
   </si>
   <si>
     <t>CI469</t>
   </si>
   <si>
+    <t>CI471</t>
+  </si>
+  <si>
+    <t>CI473</t>
+  </si>
+  <si>
     <t>REP02-0113</t>
   </si>
   <si>
+    <t>CI474</t>
+  </si>
+  <si>
+    <t>CI475</t>
+  </si>
+  <si>
+    <t>CI476</t>
+  </si>
+  <si>
+    <t>CI478</t>
+  </si>
+  <si>
+    <t>CI479</t>
+  </si>
+  <si>
+    <t>CI480</t>
+  </si>
+  <si>
+    <t>CI483</t>
+  </si>
+  <si>
+    <t>CI484</t>
+  </si>
+  <si>
+    <t>CI485</t>
+  </si>
+  <si>
+    <t>CI486</t>
+  </si>
+  <si>
+    <t>REP03-0113</t>
+  </si>
+  <si>
+    <t>CI487</t>
+  </si>
+  <si>
+    <t>CI488</t>
+  </si>
+  <si>
+    <t>CI491</t>
+  </si>
+  <si>
+    <t>CI492</t>
+  </si>
+  <si>
+    <t>CI493</t>
+  </si>
+  <si>
+    <t>CI494</t>
+  </si>
+  <si>
     <t>CI470</t>
   </si>
   <si>
-    <t>CI471</t>
-  </si>
-  <si>
     <t>CI472</t>
   </si>
   <si>
-    <t>CI474</t>
-  </si>
-  <si>
-    <t>CI475</t>
-  </si>
-  <si>
-    <t>CI476</t>
-  </si>
-  <si>
-    <t>CI479</t>
-  </si>
-  <si>
-    <t>CI480</t>
+    <t>CI489</t>
+  </si>
+  <si>
+    <t>CI477</t>
   </si>
   <si>
     <t>CI481</t>
@@ -318,49 +357,10 @@
     <t>CI482</t>
   </si>
   <si>
-    <t>REP03-0113</t>
-  </si>
-  <si>
-    <t>CI483</t>
-  </si>
-  <si>
-    <t>CI484</t>
-  </si>
-  <si>
-    <t>CI487</t>
-  </si>
-  <si>
-    <t>CI488</t>
-  </si>
-  <si>
-    <t>CI489</t>
-  </si>
-  <si>
     <t>CI490</t>
   </si>
   <si>
-    <t>CI466</t>
-  </si>
-  <si>
-    <t>CI468</t>
-  </si>
-  <si>
-    <t>CI485</t>
-  </si>
-  <si>
-    <t>CI473</t>
-  </si>
-  <si>
-    <t>CI477</t>
-  </si>
-  <si>
-    <t>CI478</t>
-  </si>
-  <si>
-    <t>CI486</t>
-  </si>
-  <si>
-    <t>CI491</t>
+    <t>CI495</t>
   </si>
   <si>
     <t>21470269</t>
@@ -855,7 +855,7 @@
     <t>2026-01-14 18:00</t>
   </si>
   <si>
-    <t>CI463: H&amp;S Daily Clean Libra</t>
+    <t>CI467: H&amp;S Daily Clean Libra</t>
   </si>
   <si>
     <t>WASHOUT</t>
@@ -864,37 +864,31 @@
     <t>REP01-0113: HC BASE</t>
   </si>
   <si>
-    <t>CI464: H&amp;S Daily Cool Libra</t>
-  </si>
-  <si>
-    <t>CI465: H&amp;S Daily Clean Libra</t>
-  </si>
-  <si>
-    <t>CI467: H&amp;S Daily Cool Libra</t>
+    <t>CI468: H&amp;S Daily Cool Libra</t>
   </si>
   <si>
     <t>CI469: H&amp;S Daily Clean Libra</t>
   </si>
   <si>
+    <t>CI471: H&amp;S Daily Cool Libra</t>
+  </si>
+  <si>
+    <t>CI473: H&amp;S Daily Clean Libra</t>
+  </si>
+  <si>
     <t>REP02-0113: HC BASE</t>
   </si>
   <si>
-    <t>CI470: PTN Silky Smooth Shampoo</t>
-  </si>
-  <si>
-    <t>CI471: H&amp;S Daily Cool Libra</t>
-  </si>
-  <si>
-    <t>CI472: H&amp;S Daily Clean Libra</t>
-  </si>
-  <si>
-    <t>CI474: H&amp;S SS</t>
-  </si>
-  <si>
-    <t>CI475: H&amp;S Daily Clean Libra</t>
-  </si>
-  <si>
-    <t>CI476: H&amp;S Daily Cool Libra</t>
+    <t>CI474: PTN Silky Smooth Shampoo</t>
+  </si>
+  <si>
+    <t>CI475: H&amp;S Daily Cool Libra</t>
+  </si>
+  <si>
+    <t>CI476: H&amp;S Daily Clean Libra</t>
+  </si>
+  <si>
+    <t>CI478: H&amp;S SS</t>
   </si>
   <si>
     <t>CI479: H&amp;S Daily Clean Libra</t>
@@ -903,58 +897,64 @@
     <t>CI480: H&amp;S Daily Cool Libra</t>
   </si>
   <si>
-    <t>CI481: H&amp;S Daily Clean Libra</t>
-  </si>
-  <si>
-    <t>CI482: H&amp;S Neem Libra</t>
+    <t>CI483: H&amp;S Daily Clean Libra</t>
+  </si>
+  <si>
+    <t>CI484: H&amp;S Daily Cool Libra</t>
+  </si>
+  <si>
+    <t>CI485: H&amp;S Daily Clean Libra</t>
+  </si>
+  <si>
+    <t>CI486: H&amp;S Neem Libra</t>
   </si>
   <si>
     <t>REP03-0113: HC BASE</t>
   </si>
   <si>
-    <t>CI483: H&amp;S SS</t>
-  </si>
-  <si>
-    <t>CI484: H&amp;S Daily Clean Libra</t>
-  </si>
-  <si>
-    <t>CI487: H&amp;S Daily Clean Libra</t>
-  </si>
-  <si>
-    <t>CI488: H&amp;S Daily Cool Libra</t>
-  </si>
-  <si>
-    <t>CI489: H&amp;S Daily Clean Libra</t>
-  </si>
-  <si>
-    <t>CI490: H&amp;S Daily Cool Libra</t>
-  </si>
-  <si>
-    <t>CI466: H&amp;S AHF 2in1</t>
-  </si>
-  <si>
-    <t>CI468: PTN Lively Clean</t>
-  </si>
-  <si>
-    <t>CI485: PTN HFC Conditioner</t>
+    <t>CI487: H&amp;S SS</t>
+  </si>
+  <si>
+    <t>CI488: H&amp;S Daily Clean Libra</t>
+  </si>
+  <si>
+    <t>CI491: H&amp;S Daily Clean Libra</t>
+  </si>
+  <si>
+    <t>CI492: H&amp;S Daily Cool Libra</t>
+  </si>
+  <si>
+    <t>CI493: H&amp;S Daily Clean Libra</t>
+  </si>
+  <si>
+    <t>CI494: H&amp;S Daily Cool Libra</t>
+  </si>
+  <si>
+    <t>CI470: H&amp;S AHF 2in1</t>
+  </si>
+  <si>
+    <t>CI472: PTN Lively Clean</t>
+  </si>
+  <si>
+    <t>CI489: PTN HFC Conditioner</t>
   </si>
   <si>
     <t>COND WASH (60m)</t>
   </si>
   <si>
-    <t>CI473: PTN  Hair Fall Control</t>
-  </si>
-  <si>
-    <t>CI477: H&amp;S AHF</t>
-  </si>
-  <si>
-    <t>CI478: H&amp;S CM</t>
-  </si>
-  <si>
-    <t>CI486: H&amp;S Neem Libra</t>
-  </si>
-  <si>
-    <t>CI491: PTN HFC Conditioner</t>
+    <t>CI477: PTN  Hair Fall Control</t>
+  </si>
+  <si>
+    <t>CI481: H&amp;S AHF</t>
+  </si>
+  <si>
+    <t>CI482: H&amp;S CM</t>
+  </si>
+  <si>
+    <t>CI490: H&amp;S Neem Libra</t>
+  </si>
+  <si>
+    <t>CI495: PTN HFC Conditioner</t>
   </si>
   <si>
     <t>Sr.No</t>
@@ -3290,16 +3290,16 @@
         <v>132</v>
       </c>
       <c r="L33" s="2">
-        <v>46035.76388888889</v>
+        <v>46035.84791666667</v>
       </c>
       <c r="M33">
         <v>90</v>
       </c>
       <c r="N33" s="2">
-        <v>46035.82638888889</v>
+        <v>46035.91041666667</v>
       </c>
       <c r="O33">
-        <v>2281</v>
+        <v>2160</v>
       </c>
       <c r="P33" t="s">
         <v>135</v>
@@ -4311,9 +4311,6 @@
       <c r="C91" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="D91" s="3" t="s">
-        <v>312</v>
-      </c>
     </row>
     <row r="92" spans="1:4">
       <c r="A92" t="s">
@@ -4325,9 +4322,6 @@
       <c r="C92" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="D92" s="3" t="s">
-        <v>312</v>
-      </c>
     </row>
     <row r="93" spans="1:4">
       <c r="A93" t="s">
@@ -4339,9 +4333,6 @@
       <c r="C93" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="D93" s="3" t="s">
-        <v>312</v>
-      </c>
     </row>
     <row r="94" spans="1:4">
       <c r="A94" t="s">
@@ -4364,6 +4355,9 @@
       <c r="C95" s="3" t="s">
         <v>298</v>
       </c>
+      <c r="D95" s="3" t="s">
+        <v>312</v>
+      </c>
     </row>
     <row r="96" spans="1:4">
       <c r="A96" t="s">
@@ -4375,8 +4369,11 @@
       <c r="C96" s="3" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="97" spans="1:3">
+      <c r="D96" s="3" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4">
       <c r="A97" t="s">
         <v>237</v>
       </c>
@@ -4386,8 +4383,11 @@
       <c r="C97" s="3" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="98" spans="1:3">
+      <c r="D97" s="3" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4">
       <c r="A98" t="s">
         <v>238</v>
       </c>
@@ -4398,7 +4398,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="99" spans="1:3">
+    <row r="99" spans="1:4">
       <c r="A99" t="s">
         <v>239</v>
       </c>
@@ -4409,7 +4409,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="100" spans="1:3">
+    <row r="100" spans="1:4">
       <c r="A100" t="s">
         <v>240</v>
       </c>
@@ -4420,7 +4420,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="101" spans="1:3">
+    <row r="101" spans="1:4">
       <c r="A101" t="s">
         <v>241</v>
       </c>
@@ -4428,7 +4428,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="102" spans="1:3">
+    <row r="102" spans="1:4">
       <c r="A102" t="s">
         <v>242</v>
       </c>
@@ -4436,7 +4436,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="103" spans="1:3">
+    <row r="103" spans="1:4">
       <c r="A103" t="s">
         <v>243</v>
       </c>
@@ -4444,7 +4444,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="104" spans="1:3">
+    <row r="104" spans="1:4">
       <c r="A104" t="s">
         <v>244</v>
       </c>
@@ -4452,7 +4452,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="105" spans="1:3">
+    <row r="105" spans="1:4">
       <c r="A105" t="s">
         <v>245</v>
       </c>
@@ -4460,7 +4460,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="106" spans="1:3">
+    <row r="106" spans="1:4">
       <c r="A106" t="s">
         <v>246</v>
       </c>
@@ -4468,7 +4468,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="107" spans="1:3">
+    <row r="107" spans="1:4">
       <c r="A107" t="s">
         <v>247</v>
       </c>
@@ -4476,7 +4476,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="108" spans="1:3">
+    <row r="108" spans="1:4">
       <c r="A108" t="s">
         <v>248</v>
       </c>
@@ -4484,7 +4484,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="109" spans="1:3">
+    <row r="109" spans="1:4">
       <c r="A109" t="s">
         <v>249</v>
       </c>
@@ -4492,7 +4492,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="110" spans="1:3">
+    <row r="110" spans="1:4">
       <c r="A110" t="s">
         <v>250</v>
       </c>
@@ -4500,7 +4500,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="111" spans="1:3">
+    <row r="111" spans="1:4">
       <c r="A111" t="s">
         <v>251</v>
       </c>
@@ -4508,7 +4508,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="112" spans="1:3">
+    <row r="112" spans="1:4">
       <c r="A112" t="s">
         <v>252</v>
       </c>

</xml_diff>